<commit_message>
update: add arguments unit test and extend xlsx tests for DAYS, DAYS360
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/DATE_AND_TIME/DAYS_DAYS360.xlsx
+++ b/xlsx/tests/calc_tests/DATE_AND_TIME/DAYS_DAYS360.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B571125E-9301-3849-BC0D-23FAC119691B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC1D8147-1BE7-4D18-B3D6-C90419CBC8DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="18580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="119">
   <si>
     <t>End date</t>
   </si>
@@ -190,6 +190,204 @@
   </si>
   <si>
     <t>Text in quotes with preceding space</t>
+  </si>
+  <si>
+    <t>EOM: start on 31st into Feb (non-leap)</t>
+  </si>
+  <si>
+    <t>EOM: start on 31st into Feb 29 (leap)</t>
+  </si>
+  <si>
+    <t>EOM: Feb 28 to Mar 31 (non-leap)</t>
+  </si>
+  <si>
+    <t>EOM: Feb 29 to Mar 31 (leap)</t>
+  </si>
+  <si>
+    <t>EOM: 31st to 31st, two months apart</t>
+  </si>
+  <si>
+    <t>EOM: 31st to 31st across a 30-day month</t>
+  </si>
+  <si>
+    <t>EOM: start on 30th, end on 30th</t>
+  </si>
+  <si>
+    <t>EOM: start 31st vs 30th, same end date</t>
+  </si>
+  <si>
+    <t>EOM: 30th to 31st within one month</t>
+  </si>
+  <si>
+    <t>EOM: full year ending on the 31st</t>
+  </si>
+  <si>
+    <t>EOM: 31st crossing the year boundary</t>
+  </si>
+  <si>
+    <t>EOM: same date, both end of a 30-day month</t>
+  </si>
+  <si>
+    <t>EOM: same date, both end of Feb</t>
+  </si>
+  <si>
+    <t>Serial boundary: max supported date</t>
+  </si>
+  <si>
+    <t>Serial boundary: one past max date</t>
+  </si>
+  <si>
+    <t>Fractional serials within the same day</t>
+  </si>
+  <si>
+    <t>Fractional serials straddling midnight</t>
+  </si>
+  <si>
+    <t>Negative fractional serials</t>
+  </si>
+  <si>
+    <t>2026-07-01</t>
+  </si>
+  <si>
+    <t>July 1, 2026</t>
+  </si>
+  <si>
+    <t>1/1/29</t>
+  </si>
+  <si>
+    <t>1/1/30</t>
+  </si>
+  <si>
+    <t>45000</t>
+  </si>
+  <si>
+    <t>2025-02-29</t>
+  </si>
+  <si>
+    <t>2026-06-01</t>
+  </si>
+  <si>
+    <t>June 1, 2026</t>
+  </si>
+  <si>
+    <t>1/1/28</t>
+  </si>
+  <si>
+    <t>44999</t>
+  </si>
+  <si>
+    <t>2025-02-01</t>
+  </si>
+  <si>
+    <t>String: ISO 8601 format</t>
+  </si>
+  <si>
+    <t>String: long month-name format</t>
+  </si>
+  <si>
+    <t>String: 2-digit year below the 2029 pivot</t>
+  </si>
+  <si>
+    <t>String: 2-digit year across the 2029/2030 pivot</t>
+  </si>
+  <si>
+    <t>String: numeric text serial</t>
+  </si>
+  <si>
+    <t>String: Feb 29 in a non-leap year</t>
+  </si>
+  <si>
+    <t>Precision: near-full day inside one calendar day</t>
+  </si>
+  <si>
+    <t>Precision: minimal span across midnight</t>
+  </si>
+  <si>
+    <t>Precision: exact half-day offsets, one day apart</t>
+  </si>
+  <si>
+    <t>Precision: just over one day, fractional both sides</t>
+  </si>
+  <si>
+    <t>Precision: reversed fractional arguments</t>
+  </si>
+  <si>
+    <t>Precision: end is whole day, start is late same day</t>
+  </si>
+  <si>
+    <t>Argument is number 1 (equivalent to TRUE)</t>
+  </si>
+  <si>
+    <t>Argument is negative 1</t>
+  </si>
+  <si>
+    <t>Argument is small negative decimal</t>
+  </si>
+  <si>
+    <t>Argument is near-zero decimal</t>
+  </si>
+  <si>
+    <t>Argument is very large number</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>Argument is lowercase text FALSE</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Argument is numeric text 1</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Argument is numeric text 0</t>
+  </si>
+  <si>
+    <t>Argument is empty text string</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Argument is a single space</t>
+  </si>
+  <si>
+    <t>Argument is boolean TRUE (European method)</t>
+  </si>
+  <si>
+    <t>Argument is boolean FALSE (US/NASD method)</t>
+  </si>
+  <si>
+    <t>Argument is number 0</t>
+  </si>
+  <si>
+    <t>Argument is number 1</t>
+  </si>
+  <si>
+    <t>Argument omitted (empty cell)</t>
+  </si>
+  <si>
+    <t>Empty first argument</t>
+  </si>
+  <si>
+    <t>Empty second argument</t>
+  </si>
+  <si>
+    <t>All arguments empty</t>
+  </si>
+  <si>
+    <t>Empty first argument (direct ref)</t>
+  </si>
+  <si>
+    <t>Empty second argument (direct ref)</t>
+  </si>
+  <si>
+    <t>All arguments empty (direct ref)</t>
   </si>
 </sst>
 </file>
@@ -230,7 +428,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -240,12 +438,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -277,7 +469,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -291,11 +483,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -577,7 +768,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="3">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -599,17 +790,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F54CD0-8216-4E1F-9732-2CE5FAC307BD}">
-  <dimension ref="A1:J44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J82"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="4" width="15.6640625" customWidth="1"/>
-    <col min="5" max="5" width="38.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="11.33203125" customWidth="1"/>
-    <col min="10" max="10" width="27.1640625" customWidth="1"/>
+    <col min="1" max="2" width="17.08984375" customWidth="1"/>
+    <col min="3" max="4" width="15.6328125" customWidth="1"/>
+    <col min="5" max="5" width="38.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.81640625" customWidth="1"/>
+    <col min="9" max="9" width="11.36328125" customWidth="1"/>
+    <col min="10" max="10" width="27.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -635,7 +827,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <f>DATE(2025,1,10)</f>
         <v>45667</v>
@@ -662,8 +854,11 @@
       <c r="I2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <f>DATE(2026,1,1)</f>
         <v>46023</v>
@@ -690,8 +885,11 @@
       <c r="I3" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <f>DATE(2025,1,1)</f>
         <v>45658</v>
@@ -722,7 +920,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <f>DATE(9990,5,12)</f>
         <v>2954945</v>
@@ -753,7 +951,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <f>DATE(2025,1,1)</f>
         <v>45658</v>
@@ -784,7 +982,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <f>DATE(2026,2,4)</f>
         <v>46057</v>
@@ -794,11 +992,11 @@
         <v>45942</v>
       </c>
       <c r="C7" s="3">
-        <f t="shared" si="0"/>
+        <f>_xlfn.DAYS(DATE(2026,2,4),DATE(2025,10,12))</f>
         <v>115</v>
       </c>
       <c r="D7" s="3">
-        <f t="shared" si="1"/>
+        <f>DAYS360(DATE(2025,10,12),DATE(2026,2,4))</f>
         <v>112</v>
       </c>
       <c r="E7" t="s">
@@ -811,8 +1009,11 @@
       <c r="I7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <f>DATE(2025,12,8)</f>
         <v>45999</v>
@@ -839,8 +1040,11 @@
       <c r="I8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <f>DATE(2025,12,8)</f>
         <v>45999</v>
@@ -864,8 +1068,11 @@
         <f t="shared" si="2"/>
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <f>DATE(2025,12,8)</f>
         <v>45999</v>
@@ -896,7 +1103,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <f>DATE(2025,12,8)</f>
         <v>45999</v>
@@ -927,7 +1134,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <f>DATE(2024,3,1)</f>
         <v>45352</v>
@@ -958,7 +1165,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <f>DATE(2024,3,1)</f>
         <v>45352</v>
@@ -989,7 +1196,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <f>DATE(2025,2,28)</f>
         <v>45716</v>
@@ -1002,7 +1209,7 @@
         <f t="shared" si="0"/>
         <v>365</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="3">
         <f t="shared" si="1"/>
         <v>358</v>
       </c>
@@ -1020,7 +1227,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <f>DATE(2025,3,1)</f>
         <v>45717</v>
@@ -1040,8 +1247,18 @@
       <c r="E15" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H15" s="3">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I15)</f>
+        <v>29</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <f>DATE(2025,7,31)</f>
         <v>45869</v>
@@ -1061,8 +1278,18 @@
       <c r="E16" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="H16" s="3">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I16)</f>
+        <v>29</v>
+      </c>
+      <c r="I16">
+        <v>-1</v>
+      </c>
+      <c r="J16" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <f>DATE(2025,7,31)</f>
         <v>45869</v>
@@ -1082,8 +1309,18 @@
       <c r="E17" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="H17" s="3">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I17)</f>
+        <v>29</v>
+      </c>
+      <c r="I17">
+        <v>-1E-4</v>
+      </c>
+      <c r="J17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <f>DATE(2024,2,28)</f>
         <v>45350</v>
@@ -1103,8 +1340,18 @@
       <c r="E18" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="H18" s="3">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I18)</f>
+        <v>29</v>
+      </c>
+      <c r="I18">
+        <v>1.0000000000000001E-15</v>
+      </c>
+      <c r="J18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <f>DATE(2025,1,13)</f>
         <v>45670</v>
@@ -1124,8 +1371,18 @@
       <c r="E19" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="H19" s="3">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I19)</f>
+        <v>29</v>
+      </c>
+      <c r="I19">
+        <v>1000000</v>
+      </c>
+      <c r="J19" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <f>DATE(2025,1,10)+TIME(23,59,0)</f>
         <v>45667.999305555553</v>
@@ -1145,8 +1402,18 @@
       <c r="E20" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="H20" s="3">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I20)</f>
+        <v>30</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="J20" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <f>DATE(2025,1,14)+TIME(0,1,0)</f>
         <v>45671.000694444447</v>
@@ -1166,8 +1433,18 @@
       <c r="E21" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="H21" s="3" t="e">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I21)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I21" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="J21" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>9</v>
       </c>
@@ -1185,8 +1462,18 @@
       <c r="E22" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="H22" s="3" t="e">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I22)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="J22" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>46000</v>
       </c>
@@ -1205,27 +1492,45 @@
       <c r="E23" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="10">
+      <c r="H23" s="3">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I23)</f>
+        <v>30</v>
+      </c>
+      <c r="I23" s="11"/>
+      <c r="J23" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="9">
         <v>46000.999999</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="9">
         <v>45992.000001</v>
       </c>
       <c r="C24" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="3">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="E24" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="H24" s="3" t="e">
+        <f>DAYS360(DATE(2025,1,1),DATE(2025,1,31),I24)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="J24" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>-5</v>
       </c>
@@ -1244,18 +1549,18 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>1</v>
       </c>
       <c r="B26">
         <v>0</v>
       </c>
-      <c r="C26" s="9">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="D26" s="9">
+      <c r="C26" s="3">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D26" s="3">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -1263,18 +1568,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>10</v>
       </c>
       <c r="B27">
         <v>0</v>
       </c>
-      <c r="C27" s="9">
+      <c r="C27" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="3">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -1282,15 +1587,15 @@
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>10</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D28" s="9">
+      <c r="D28" s="3">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -1298,15 +1603,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B29">
         <v>10</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="3">
         <f t="shared" si="0"/>
         <v>-10</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="3">
         <f t="shared" si="1"/>
         <v>-10</v>
       </c>
@@ -1314,7 +1619,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
@@ -1335,7 +1640,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
@@ -1355,7 +1660,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>10</v>
       </c>
@@ -1372,12 +1677,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A33" s="11">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="10">
         <f>DATE(2025,10,1)</f>
         <v>45931</v>
       </c>
-      <c r="B33" s="11">
+      <c r="B33" s="10">
         <f>DATE(2025,1,7)</f>
         <v>45664</v>
       </c>
@@ -1393,8 +1698,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="11">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="10">
         <f>DATE(2025,10,1)</f>
         <v>45931</v>
       </c>
@@ -1407,8 +1712,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="11">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="10">
         <f>DATE(2025,10,1)</f>
         <v>45931</v>
       </c>
@@ -1421,7 +1726,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>10</v>
       </c>
@@ -1440,18 +1745,18 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="b">
         <v>1</v>
       </c>
       <c r="B37" t="b">
         <v>0</v>
       </c>
-      <c r="C37" s="9">
+      <c r="C37" s="3">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="3">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -1459,15 +1764,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="b">
         <v>1</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="3">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="3">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -1475,15 +1780,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="b">
         <v>0</v>
       </c>
-      <c r="C39" s="9">
+      <c r="C39" s="3">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="D39" s="9">
+      <c r="D39" s="3">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -1491,15 +1796,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B40" t="b">
         <v>1</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="3">
         <f t="shared" si="3"/>
         <v>-1</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="3">
         <f t="shared" si="4"/>
         <v>-1</v>
       </c>
@@ -1510,15 +1815,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B41" t="b">
         <v>0</v>
       </c>
-      <c r="C41" s="9">
+      <c r="C41" s="3">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="D41" s="9">
+      <c r="D41" s="3">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -1529,7 +1834,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>5</v>
       </c>
@@ -1551,7 +1856,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>10</v>
       </c>
@@ -1573,7 +1878,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44">
         <f>1.05*(0.0284+0.0046)-0.0284</f>
         <v>6.2499999999999986E-3</v>
@@ -1581,11 +1886,11 @@
       <c r="B44">
         <v>1</v>
       </c>
-      <c r="C44" s="9">
+      <c r="C44" s="3">
         <f>_xlfn.DAYS(A44,B44)</f>
         <v>-1</v>
       </c>
-      <c r="D44" s="9">
+      <c r="D44" s="3">
         <f>DAYS360(B44,A44)</f>
         <v>-1</v>
       </c>
@@ -1594,6 +1899,731 @@
       </c>
       <c r="F44">
         <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="4">
+        <f>DATE(2025,2,28)</f>
+        <v>45716</v>
+      </c>
+      <c r="B46" s="4">
+        <f>DATE(2025,1,31)</f>
+        <v>45688</v>
+      </c>
+      <c r="C46" s="3">
+        <f>_xlfn.DAYS(A46,B46)</f>
+        <v>28</v>
+      </c>
+      <c r="D46" s="3">
+        <f>DAYS360(B46,A46)</f>
+        <v>28</v>
+      </c>
+      <c r="E46" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" s="4">
+        <f>DATE(2024,2,29)</f>
+        <v>45351</v>
+      </c>
+      <c r="B47" s="4">
+        <f>DATE(2024,1,31)</f>
+        <v>45322</v>
+      </c>
+      <c r="C47" s="3">
+        <f>_xlfn.DAYS(A47,B47)</f>
+        <v>29</v>
+      </c>
+      <c r="D47" s="3">
+        <f>DAYS360(B47,A47)</f>
+        <v>29</v>
+      </c>
+      <c r="E47" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" s="4">
+        <f>DATE(2025,3,31)</f>
+        <v>45747</v>
+      </c>
+      <c r="B48" s="4">
+        <f>DATE(2025,2,28)</f>
+        <v>45716</v>
+      </c>
+      <c r="C48" s="3">
+        <f>_xlfn.DAYS(A48,B48)</f>
+        <v>31</v>
+      </c>
+      <c r="D48" s="3">
+        <f>DAYS360(B48,A48)</f>
+        <v>30</v>
+      </c>
+      <c r="E48" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" s="4">
+        <f>DATE(2024,3,31)</f>
+        <v>45382</v>
+      </c>
+      <c r="B49" s="4">
+        <f>DATE(2024,2,29)</f>
+        <v>45351</v>
+      </c>
+      <c r="C49" s="3">
+        <f>_xlfn.DAYS(A49,B49)</f>
+        <v>31</v>
+      </c>
+      <c r="D49" s="3">
+        <f>DAYS360(B49,A49)</f>
+        <v>30</v>
+      </c>
+      <c r="E49" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" s="4">
+        <f>DATE(2025,3,31)</f>
+        <v>45747</v>
+      </c>
+      <c r="B50" s="4">
+        <f>DATE(2025,1,31)</f>
+        <v>45688</v>
+      </c>
+      <c r="C50" s="3">
+        <f>_xlfn.DAYS(A50,B50)</f>
+        <v>59</v>
+      </c>
+      <c r="D50" s="3">
+        <f>DAYS360(B50,A50)</f>
+        <v>60</v>
+      </c>
+      <c r="E50" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" s="4">
+        <f>DATE(2025,5,31)</f>
+        <v>45808</v>
+      </c>
+      <c r="B51" s="4">
+        <f>DATE(2025,3,31)</f>
+        <v>45747</v>
+      </c>
+      <c r="C51" s="3">
+        <f>_xlfn.DAYS(A51,B51)</f>
+        <v>61</v>
+      </c>
+      <c r="D51" s="3">
+        <f>DAYS360(B51,A51)</f>
+        <v>60</v>
+      </c>
+      <c r="E51" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" s="4">
+        <f>DATE(2025,4,30)</f>
+        <v>45777</v>
+      </c>
+      <c r="B52" s="4">
+        <f>DATE(2025,1,30)</f>
+        <v>45687</v>
+      </c>
+      <c r="C52" s="3">
+        <f>_xlfn.DAYS(A52,B52)</f>
+        <v>90</v>
+      </c>
+      <c r="D52" s="3">
+        <f>DAYS360(B52,A52)</f>
+        <v>90</v>
+      </c>
+      <c r="E52" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" s="4">
+        <f>DATE(2025,4,30)</f>
+        <v>45777</v>
+      </c>
+      <c r="B53" s="4">
+        <f>DATE(2025,1,31)</f>
+        <v>45688</v>
+      </c>
+      <c r="C53" s="3">
+        <f>_xlfn.DAYS(A53,B53)</f>
+        <v>89</v>
+      </c>
+      <c r="D53" s="3">
+        <f>DAYS360(B53,A53)</f>
+        <v>90</v>
+      </c>
+      <c r="E53" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54" s="4">
+        <f>DATE(2025,1,31)</f>
+        <v>45688</v>
+      </c>
+      <c r="B54" s="4">
+        <f>DATE(2025,1,30)</f>
+        <v>45687</v>
+      </c>
+      <c r="C54" s="3">
+        <f>_xlfn.DAYS(A54,B54)</f>
+        <v>1</v>
+      </c>
+      <c r="D54" s="3">
+        <f>DAYS360(B54,A54)</f>
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" s="4">
+        <f>DATE(2025,12,31)</f>
+        <v>46022</v>
+      </c>
+      <c r="B55" s="4">
+        <f>DATE(2025,1,1)</f>
+        <v>45658</v>
+      </c>
+      <c r="C55" s="3">
+        <f>_xlfn.DAYS(A55,B55)</f>
+        <v>364</v>
+      </c>
+      <c r="D55" s="3">
+        <f>DAYS360(B55,A55)</f>
+        <v>360</v>
+      </c>
+      <c r="E55" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" s="4">
+        <f>DATE(2026,1,1)</f>
+        <v>46023</v>
+      </c>
+      <c r="B56" s="4">
+        <f>DATE(2025,12,31)</f>
+        <v>46022</v>
+      </c>
+      <c r="C56" s="3">
+        <f>_xlfn.DAYS(A56,B56)</f>
+        <v>1</v>
+      </c>
+      <c r="D56" s="3">
+        <f>DAYS360(B56,A56)</f>
+        <v>1</v>
+      </c>
+      <c r="E56" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A57" s="4">
+        <f>DATE(2025,6,30)</f>
+        <v>45838</v>
+      </c>
+      <c r="B57" s="4">
+        <f>DATE(2025,6,30)</f>
+        <v>45838</v>
+      </c>
+      <c r="C57" s="3">
+        <f>_xlfn.DAYS(A57,B57)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="3">
+        <f>DAYS360(B57,A57)</f>
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" s="4">
+        <f>DATE(2025,2,28)</f>
+        <v>45716</v>
+      </c>
+      <c r="B58" s="4">
+        <f>DATE(2025,2,28)</f>
+        <v>45716</v>
+      </c>
+      <c r="C58" s="3">
+        <f>_xlfn.DAYS(A58,B58)</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="3">
+        <f>DAYS360(B58,A58)</f>
+        <v>-2</v>
+      </c>
+      <c r="E58" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" s="4">
+        <f>DATE(9999,12,31)</f>
+        <v>2958465</v>
+      </c>
+      <c r="B59" s="4">
+        <f>DATE(9999,12,30)</f>
+        <v>2958464</v>
+      </c>
+      <c r="C59" s="3">
+        <f>_xlfn.DAYS(A59,B59)</f>
+        <v>1</v>
+      </c>
+      <c r="D59" s="3">
+        <f>DAYS360(B59,A59)</f>
+        <v>0</v>
+      </c>
+      <c r="E59" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" s="12">
+        <v>2958466</v>
+      </c>
+      <c r="B60" s="4">
+        <f>DATE(9999,12,31)</f>
+        <v>2958465</v>
+      </c>
+      <c r="C60" s="3" t="e">
+        <f>_xlfn.DAYS(A60,B60)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="D60" s="3" t="e">
+        <f>DAYS360(B60,A60)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E60" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" s="4">
+        <f>DATE(2025,1,1)+0.9999</f>
+        <v>45658.999900000003</v>
+      </c>
+      <c r="B61" s="4">
+        <f>DATE(2025,1,1)+0.0001</f>
+        <v>45658.000099999997</v>
+      </c>
+      <c r="C61" s="3">
+        <f>_xlfn.DAYS(A61,B61)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="3">
+        <f>DAYS360(B61,A61)</f>
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" s="4">
+        <f>DATE(2025,1,2)+0.4</f>
+        <v>45659.4</v>
+      </c>
+      <c r="B62" s="4">
+        <f>DATE(2025,1,1)+0.6</f>
+        <v>45658.6</v>
+      </c>
+      <c r="C62" s="3">
+        <f>_xlfn.DAYS(A62,B62)</f>
+        <v>1</v>
+      </c>
+      <c r="D62" s="3">
+        <f>DAYS360(B62,A62)</f>
+        <v>1</v>
+      </c>
+      <c r="E62" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" s="12">
+        <f>-(DATE(2025,1,1)+0.5)</f>
+        <v>-45658.5</v>
+      </c>
+      <c r="B63" s="12">
+        <f>-(DATE(2025,1,2)+0.5)</f>
+        <v>-45659.5</v>
+      </c>
+      <c r="C63" s="3" t="e">
+        <f>_xlfn.DAYS(A63,B63)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="D63" s="3" t="e">
+        <f>DAYS360(B63,A63)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E63" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64" s="4"/>
+      <c r="B64" s="4">
+        <f>DATE(2025,1,1)</f>
+        <v>45658</v>
+      </c>
+      <c r="C64" s="3">
+        <f t="shared" ref="C64:C66" si="5">_xlfn.DAYS(A64,B64)</f>
+        <v>-45658</v>
+      </c>
+      <c r="D64" s="3">
+        <f t="shared" ref="D64:D66" si="6">DAYS360(B64,A64)</f>
+        <v>-45001</v>
+      </c>
+      <c r="E64" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65" s="4">
+        <f t="shared" ref="A65:A68" si="7">DATE(2025,1,10)</f>
+        <v>45667</v>
+      </c>
+      <c r="B65" s="4"/>
+      <c r="C65" s="3">
+        <f t="shared" si="5"/>
+        <v>45667</v>
+      </c>
+      <c r="D65" s="3">
+        <f t="shared" si="6"/>
+        <v>45010</v>
+      </c>
+      <c r="E65" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66" s="4"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="3">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D66" s="3">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67" s="4"/>
+      <c r="B67" s="4">
+        <f>DATE(2025,1,1)</f>
+        <v>45658</v>
+      </c>
+      <c r="C67" s="3">
+        <f>_xlfn.DAYS(,B67)</f>
+        <v>-45658</v>
+      </c>
+      <c r="D67" s="3">
+        <f>DAYS360(,B67)</f>
+        <v>45001</v>
+      </c>
+      <c r="E67" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A68" s="4">
+        <f t="shared" si="7"/>
+        <v>45667</v>
+      </c>
+      <c r="B68" s="4"/>
+      <c r="C68" s="3">
+        <f>_xlfn.DAYS(A68,)</f>
+        <v>45667</v>
+      </c>
+      <c r="D68" s="3">
+        <f>DAYS360(A68,)</f>
+        <v>-45010</v>
+      </c>
+      <c r="E68" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69" s="4"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="3">
+        <f>_xlfn.DAYS(,)</f>
+        <v>0</v>
+      </c>
+      <c r="D69" s="3">
+        <f>DAYS360(,)</f>
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C70" s="3">
+        <f>_xlfn.DAYS(A70,B70)</f>
+        <v>30</v>
+      </c>
+      <c r="D70" s="3">
+        <f>DAYS360(B70,A70)</f>
+        <v>30</v>
+      </c>
+      <c r="E70" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="C71" s="3" t="e">
+        <f>_xlfn.DAYS(A71,B71)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D71" s="3" t="e">
+        <f>DAYS360(B71,A71)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E71" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A72" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="C72" s="3">
+        <f>_xlfn.DAYS(A72,B72)</f>
+        <v>366</v>
+      </c>
+      <c r="D72" s="3">
+        <f>DAYS360(B72,A72)</f>
+        <v>360</v>
+      </c>
+      <c r="E72" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B73" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C73" s="3">
+        <f>_xlfn.DAYS(A73,B73)</f>
+        <v>-36160</v>
+      </c>
+      <c r="D73" s="3">
+        <f>DAYS360(B73,A73)</f>
+        <v>-35640</v>
+      </c>
+      <c r="E73" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C74" s="3">
+        <f>_xlfn.DAYS(A74,B74)</f>
+        <v>1</v>
+      </c>
+      <c r="D74" s="3">
+        <f>DAYS360(B74,A74)</f>
+        <v>1</v>
+      </c>
+      <c r="E74" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A75" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B75" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C75" s="3" t="e">
+        <f>_xlfn.DAYS(A75,B75)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D75" s="3" t="e">
+        <f>DAYS360(B75,A75)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E75" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A76" s="4"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="3"/>
+      <c r="D76" s="3"/>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A77" s="4">
+        <f>DATE(2025,1,1)+0.9999999</f>
+        <v>45658.999999899999</v>
+      </c>
+      <c r="B77" s="4">
+        <f>DATE(2025,1,1)+0.0000001</f>
+        <v>45658.000000100001</v>
+      </c>
+      <c r="C77" s="3">
+        <f>_xlfn.DAYS(A77,B77)</f>
+        <v>0</v>
+      </c>
+      <c r="D77" s="3">
+        <f>DAYS360(B77,A77)</f>
+        <v>1</v>
+      </c>
+      <c r="E77" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A78" s="4">
+        <f>DATE(2025,1,2)+0.0000001</f>
+        <v>45659.000000100001</v>
+      </c>
+      <c r="B78" s="4">
+        <f>DATE(2025,1,1)+0.9999999</f>
+        <v>45658.999999899999</v>
+      </c>
+      <c r="C78" s="3">
+        <f>_xlfn.DAYS(A78,B78)</f>
+        <v>1</v>
+      </c>
+      <c r="D78" s="3">
+        <f>DAYS360(B78,A78)</f>
+        <v>0</v>
+      </c>
+      <c r="E78" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A79" s="4">
+        <f>DATE(2025,1,2)+0.5</f>
+        <v>45659.5</v>
+      </c>
+      <c r="B79" s="4">
+        <f>DATE(2025,1,1)+0.5</f>
+        <v>45658.5</v>
+      </c>
+      <c r="C79" s="3">
+        <f>_xlfn.DAYS(A79,B79)</f>
+        <v>1</v>
+      </c>
+      <c r="D79" s="3">
+        <f>DAYS360(B79,A79)</f>
+        <v>1</v>
+      </c>
+      <c r="E79" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A80" s="4">
+        <f>DATE(2025,1,2)+0.5</f>
+        <v>45659.5</v>
+      </c>
+      <c r="B80" s="4">
+        <f>DATE(2025,1,1)+0.4999999</f>
+        <v>45658.499999899999</v>
+      </c>
+      <c r="C80" s="3">
+        <f>_xlfn.DAYS(A80,B80)</f>
+        <v>1</v>
+      </c>
+      <c r="D80" s="3">
+        <f>DAYS360(B80,A80)</f>
+        <v>1</v>
+      </c>
+      <c r="E80" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A81" s="4">
+        <f>DATE(2025,1,1)+0.5</f>
+        <v>45658.5</v>
+      </c>
+      <c r="B81" s="4">
+        <f>DATE(2025,1,2)+0.5</f>
+        <v>45659.5</v>
+      </c>
+      <c r="C81" s="3">
+        <f>_xlfn.DAYS(A81,B81)</f>
+        <v>-1</v>
+      </c>
+      <c r="D81" s="3">
+        <f>DAYS360(B81,A81)</f>
+        <v>-1</v>
+      </c>
+      <c r="E81" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A82" s="4">
+        <f>DATE(2025,1,1)</f>
+        <v>45658</v>
+      </c>
+      <c r="B82" s="4">
+        <f>DATE(2025,1,1)+0.9999999</f>
+        <v>45658.999999899999</v>
+      </c>
+      <c r="C82" s="3">
+        <f>_xlfn.DAYS(A82,B82)</f>
+        <v>0</v>
+      </c>
+      <c r="D82" s="3">
+        <f>DAYS360(B82,A82)</f>
+        <v>-1</v>
+      </c>
+      <c r="E82" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>